<commit_message>
Added NBTs to repo for 7 towns, Lycaeum, and InsideMoongate.  Britan needs to be redone.
Britain - needs named banner (red).   and NPCs had lost their tags when I checked earlier.
</commit_message>
<xml_diff>
--- a/spoilers/Ultima_IV_NPC_Dialogue_COMPLETE-with-MC.xlsx
+++ b/spoilers/Ultima_IV_NPC_Dialogue_COMPLETE-with-MC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D7D4DC-34B3-4F64-84D6-71000C0693F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A09859-48BF-46DA-A13D-9371047369AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" tabRatio="728" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" tabRatio="728" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NPC Dialogue" sheetId="1" r:id="rId1"/>
@@ -7917,9 +7917,6 @@
   </si>
   <si>
     <t>At the Inn; a cartographer</t>
-  </si>
-  <si>
-    <t>Has two of the three metallurgists</t>
   </si>
   <si>
     <t>FEAR</t>
@@ -8248,6 +8245,9 @@
   </si>
   <si>
     <t>We just got the new wainscotting.  It's OK.  We wallpapered over that hole.</t>
+  </si>
+  <si>
+    <t>Has 1-2 of the three metallurgists</t>
   </si>
 </sst>
 </file>
@@ -8603,7 +8603,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -8793,23 +8793,6 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -29999,7 +29982,7 @@
         <v>1040</v>
       </c>
       <c r="E601" s="2" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="F601" s="2" t="s">
         <v>1051</v>
@@ -30742,13 +30725,13 @@
       <c r="C622" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D622" s="75" t="s">
+      <c r="D622" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E622" s="75" t="s">
+      <c r="E622" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F622" s="75" t="s">
+      <c r="F622" s="2" t="s">
         <v>93</v>
       </c>
       <c r="G622" s="8" t="str">
@@ -30777,13 +30760,13 @@
       <c r="C623" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D623" s="75" t="s">
+      <c r="D623" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E623" s="75" t="s">
+      <c r="E623" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F623" s="75" t="s">
+      <c r="F623" s="2" t="s">
         <v>293</v>
       </c>
       <c r="G623" s="8" t="str">
@@ -30812,13 +30795,13 @@
       <c r="C624" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D624" s="75" t="s">
+      <c r="D624" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E624" s="75" t="s">
+      <c r="E624" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F624" s="75" t="s">
+      <c r="F624" s="2" t="s">
         <v>292</v>
       </c>
       <c r="G624" s="8" t="str">
@@ -30847,13 +30830,13 @@
       <c r="C625" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D625" s="75" t="s">
+      <c r="D625" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E625" s="75" t="s">
+      <c r="E625" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F625" s="75" t="s">
+      <c r="F625" s="2" t="s">
         <v>288</v>
       </c>
       <c r="G625" s="8" t="str">
@@ -30882,13 +30865,13 @@
       <c r="C626" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D626" s="75" t="s">
+      <c r="D626" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E626" s="75" t="s">
+      <c r="E626" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="F626" s="75" t="s">
+      <c r="F626" s="2" t="s">
         <v>296</v>
       </c>
       <c r="G626" s="8" t="str">
@@ -30917,14 +30900,14 @@
       <c r="C627" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D627" s="75" t="s">
+      <c r="D627" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E627" s="75" t="s">
+      <c r="E627" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="F627" s="75" t="s">
-        <v>2643</v>
+      <c r="F627" s="2" t="s">
+        <v>2642</v>
       </c>
       <c r="G627" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B627&amp;"|"&amp;C627&amp;"|"&amp;D627&amp;"|"&amp;E627,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -31162,13 +31145,13 @@
       <c r="C634" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D634" s="75" t="s">
+      <c r="D634" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="E634" s="75" t="s">
+      <c r="E634" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F634" s="75" t="s">
+      <c r="F634" s="2" t="s">
         <v>322</v>
       </c>
       <c r="G634" s="8" t="str">
@@ -31199,13 +31182,13 @@
       <c r="C635" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D635" s="75" t="s">
+      <c r="D635" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="E635" s="75" t="s">
+      <c r="E635" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F635" s="75" t="s">
+      <c r="F635" s="2" t="s">
         <v>321</v>
       </c>
       <c r="G635" s="8" t="str">
@@ -31236,13 +31219,13 @@
       <c r="C636" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D636" s="75" t="s">
+      <c r="D636" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="E636" s="75" t="s">
+      <c r="E636" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="F636" s="75" t="s">
+      <c r="F636" s="2" t="s">
         <v>325</v>
       </c>
       <c r="G636" s="8" t="str">
@@ -31273,13 +31256,13 @@
       <c r="C637" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D637" s="75" t="s">
+      <c r="D637" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="E637" s="75" t="s">
+      <c r="E637" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F637" s="75" t="s">
+      <c r="F637" s="2" t="s">
         <v>320</v>
       </c>
       <c r="G637" s="8" t="str">
@@ -31310,13 +31293,13 @@
       <c r="C638" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D638" s="75" t="s">
+      <c r="D638" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="E638" s="75" t="s">
+      <c r="E638" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F638" s="75" t="s">
+      <c r="F638" s="2" t="s">
         <v>316</v>
       </c>
       <c r="G638" s="8" t="str">
@@ -31347,13 +31330,13 @@
       <c r="C639" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D639" s="75" t="s">
+      <c r="D639" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="E639" s="75" t="s">
+      <c r="E639" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="F639" s="76" t="s">
+      <c r="F639" s="3" t="s">
         <v>324</v>
       </c>
       <c r="G639" s="8" t="str">
@@ -31391,7 +31374,7 @@
         <v>305</v>
       </c>
       <c r="F640" s="3" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
       <c r="G640" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B640&amp;"|"&amp;C640&amp;"|"&amp;D640&amp;"|"&amp;E640,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -32301,7 +32284,7 @@
         <v>406</v>
       </c>
       <c r="F666" s="3" t="s">
-        <v>2636</v>
+        <v>2635</v>
       </c>
       <c r="G666" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B666&amp;"|"&amp;C666&amp;"|"&amp;D666&amp;"|"&amp;E666,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -33001,7 +32984,7 @@
         <v>285</v>
       </c>
       <c r="F686" s="2" t="s">
-        <v>2642</v>
+        <v>2641</v>
       </c>
       <c r="G686" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B686&amp;"|"&amp;C686&amp;"|"&amp;D686&amp;"|"&amp;E686,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -33065,7 +33048,7 @@
         <v>277</v>
       </c>
       <c r="D688" s="2" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="E688" s="2" t="s">
         <v>386</v>
@@ -33100,7 +33083,7 @@
         <v>277</v>
       </c>
       <c r="D689" s="2" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="E689" s="2" t="s">
         <v>388</v>
@@ -33135,7 +33118,7 @@
         <v>277</v>
       </c>
       <c r="D690" s="2" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="E690" s="2" t="s">
         <v>20</v>
@@ -33170,7 +33153,7 @@
         <v>277</v>
       </c>
       <c r="D691" s="2" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="E691" s="2" t="s">
         <v>18</v>
@@ -33205,7 +33188,7 @@
         <v>277</v>
       </c>
       <c r="D692" s="2" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="E692" s="2" t="s">
         <v>16</v>
@@ -33240,13 +33223,13 @@
         <v>277</v>
       </c>
       <c r="D693" s="2" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="E693" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F693" s="2" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="G693" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B693&amp;"|"&amp;C693&amp;"|"&amp;D693&amp;"|"&amp;E693,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -34067,7 +34050,7 @@
       </c>
       <c r="K717" s="2"/>
     </row>
-    <row r="718" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="718" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A718" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Banter|HEALTH</v>
@@ -34102,7 +34085,7 @@
       </c>
       <c r="K718" s="2"/>
     </row>
-    <row r="719" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="719" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A719" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Banter|HORN</v>
@@ -34137,7 +34120,7 @@
       </c>
       <c r="K719" s="2"/>
     </row>
-    <row r="720" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="720" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A720" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Banter|JOB</v>
@@ -34172,7 +34155,7 @@
       </c>
       <c r="K720" s="2"/>
     </row>
-    <row r="721" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="721" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A721" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Banter|LOOK</v>
@@ -34207,7 +34190,7 @@
       </c>
       <c r="K721" s="2"/>
     </row>
-    <row r="722" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="722" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A722" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Banter|NAME</v>
@@ -34242,7 +34225,7 @@
       </c>
       <c r="K722" s="2"/>
     </row>
-    <row r="723" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="723" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A723" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Banter|SHRI</v>
@@ -34277,7 +34260,7 @@
       </c>
       <c r="K723" s="2"/>
     </row>
-    <row r="724" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="724" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A724" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Boozer|HEALTH</v>
@@ -34312,7 +34295,7 @@
       </c>
       <c r="K724" s="2"/>
     </row>
-    <row r="725" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="725" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A725" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Boozer|JOB</v>
@@ -34347,7 +34330,7 @@
       </c>
       <c r="K725" s="2"/>
     </row>
-    <row r="726" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="726" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A726" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Boozer|LOOK</v>
@@ -34382,7 +34365,7 @@
       </c>
       <c r="K726" s="2"/>
     </row>
-    <row r="727" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="727" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A727" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Boozer|MERC</v>
@@ -34417,7 +34400,7 @@
       </c>
       <c r="K727" s="2"/>
     </row>
-    <row r="728" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="728" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A728" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Boozer|NAME</v>
@@ -34452,7 +34435,7 @@
       </c>
       <c r="K728" s="2"/>
     </row>
-    <row r="729" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="729" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A729" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Boozer|POWE</v>
@@ -34487,7 +34470,7 @@
       </c>
       <c r="K729" s="2"/>
     </row>
-    <row r="730" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="730" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A730" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Bulbous|HEALTH</v>
@@ -34522,7 +34505,7 @@
       </c>
       <c r="K730" s="2"/>
     </row>
-    <row r="731" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="731" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A731" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Bulbous|JOB</v>
@@ -34557,7 +34540,7 @@
       </c>
       <c r="K731" s="2"/>
     </row>
-    <row r="732" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="732" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A732" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Bulbous|LOOK</v>
@@ -34592,7 +34575,7 @@
       </c>
       <c r="K732" s="2"/>
     </row>
-    <row r="733" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="733" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A733" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Bulbous|NAME</v>
@@ -34627,7 +34610,7 @@
       </c>
       <c r="K733" s="2"/>
     </row>
-    <row r="734" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="734" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A734" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Bulbous|SHOP</v>
@@ -34662,7 +34645,7 @@
       </c>
       <c r="K734" s="2"/>
     </row>
-    <row r="735" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="735" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A735" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Bulbous|SPOI</v>
@@ -34697,7 +34680,7 @@
       </c>
       <c r="K735" s="2"/>
     </row>
-    <row r="736" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="736" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A736" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Casperin|HAUN</v>
@@ -34732,7 +34715,7 @@
       </c>
       <c r="K736" s="2"/>
     </row>
-    <row r="737" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="737" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A737" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Casperin|HEALTH</v>
@@ -34767,7 +34750,7 @@
       </c>
       <c r="K737" s="2"/>
     </row>
-    <row r="738" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="738" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A738" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Casperin|JOB</v>
@@ -34802,7 +34785,7 @@
       </c>
       <c r="K738" s="2"/>
     </row>
-    <row r="739" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="739" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A739" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Casperin|LOOK</v>
@@ -34837,7 +34820,7 @@
       </c>
       <c r="K739" s="2"/>
     </row>
-    <row r="740" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="740" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A740" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Casperin|NAME</v>
@@ -34872,7 +34855,7 @@
       </c>
       <c r="K740" s="2"/>
     </row>
-    <row r="741" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="741" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A741" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Casperin|PRID</v>
@@ -34907,7 +34890,7 @@
       </c>
       <c r="K741" s="2"/>
     </row>
-    <row r="742" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="742" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A742" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Demitry|BONE</v>
@@ -34942,7 +34925,7 @@
       </c>
       <c r="K742" s="2"/>
     </row>
-    <row r="743" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="743" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A743" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Demitry|HEALTH</v>
@@ -34977,7 +34960,7 @@
       </c>
       <c r="K743" s="2"/>
     </row>
-    <row r="744" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="744" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A744" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Demitry|HORN</v>
@@ -35012,7 +34995,7 @@
       </c>
       <c r="K744" s="2"/>
     </row>
-    <row r="745" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="745" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A745" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Demitry|JOB</v>
@@ -35047,7 +35030,7 @@
       </c>
       <c r="K745" s="2"/>
     </row>
-    <row r="746" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="746" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A746" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Demitry|LOOK</v>
@@ -35082,7 +35065,7 @@
       </c>
       <c r="K746" s="2"/>
     </row>
-    <row r="747" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="747" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A747" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Demitry|NAME</v>
@@ -35117,7 +35100,7 @@
       </c>
       <c r="K747" s="2"/>
     </row>
-    <row r="748" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="748" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A748" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Faultless|HANG</v>
@@ -35154,7 +35137,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="749" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="749" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A749" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Faultless|HEALTH</v>
@@ -35191,7 +35174,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="750" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="750" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A750" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Faultless|JOB</v>
@@ -35228,7 +35211,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="751" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="751" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A751" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Faultless|LOOK</v>
@@ -35265,7 +35248,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="752" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="752" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A752" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Faultless|MANT</v>
@@ -35302,7 +35285,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="753" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="753" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A753" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Faultless|NAME</v>
@@ -35339,7 +35322,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="754" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="754" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A754" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Ghostly|HEALTH</v>
@@ -35368,7 +35351,7 @@
       <c r="J754" s="2"/>
       <c r="K754" s="2"/>
     </row>
-    <row r="755" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="755" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A755" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Ghostly|JOB</v>
@@ -35397,7 +35380,7 @@
       <c r="J755" s="2"/>
       <c r="K755" s="2"/>
     </row>
-    <row r="756" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="756" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A756" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Ghostly|LOOK</v>
@@ -35426,7 +35409,7 @@
       <c r="J756" s="2"/>
       <c r="K756" s="2"/>
     </row>
-    <row r="757" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="757" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A757" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Ghostly|NAME</v>
@@ -35455,7 +35438,7 @@
       <c r="J757" s="2"/>
       <c r="K757" s="2"/>
     </row>
-    <row r="758" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="758" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A758" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Ghostly|PEAC</v>
@@ -35484,7 +35467,7 @@
       <c r="J758" s="2"/>
       <c r="K758" s="2"/>
     </row>
-    <row r="759" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="759" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A759" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Ghostly|SPIR</v>
@@ -35513,7 +35496,7 @@
       <c r="J759" s="2"/>
       <c r="K759" s="2"/>
     </row>
-    <row r="760" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="760" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A760" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Heywood|HAUN</v>
@@ -35550,7 +35533,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="761" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="761" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A761" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Heywood|HEALTH</v>
@@ -35587,7 +35570,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="762" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="762" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A762" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Heywood|JOB</v>
@@ -35624,7 +35607,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="763" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="763" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A763" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Heywood|LOOK</v>
@@ -35661,7 +35644,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="764" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="764" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A764" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Heywood|MANT</v>
@@ -35698,7 +35681,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="765" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="765" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A765" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Heywood|NAME</v>
@@ -35735,7 +35718,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="766" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="766" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A766" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Katrina|HEALTH</v>
@@ -35772,7 +35755,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="767" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="767" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A767" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Katrina|JOB</v>
@@ -35809,7 +35792,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="768" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="768" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A768" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Katrina|LOOK</v>
@@ -35846,7 +35829,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="769" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="769" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A769" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Katrina|NAME</v>
@@ -35883,7 +35866,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="770" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="770" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A770" t="str">
         <f t="shared" si="11"/>
         <v>Magincia|Katrina|PRID</v>
@@ -35920,7 +35903,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="771" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="771" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A771" t="str">
         <f t="shared" ref="A771:A834" si="12">C771&amp;"|"&amp;D771&amp;"|"&amp;E771</f>
         <v>Magincia|Katrina|SURV</v>
@@ -35957,7 +35940,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="772" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="772" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A772" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Nate the Snake|HEALTH</v>
@@ -35986,7 +35969,7 @@
       <c r="J772" s="2"/>
       <c r="K772" s="2"/>
     </row>
-    <row r="773" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="773" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A773" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Nate the Snake|JOB</v>
@@ -36015,7 +35998,7 @@
       <c r="J773" s="2"/>
       <c r="K773" s="2"/>
     </row>
-    <row r="774" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="774" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A774" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Nate the Snake|LOOK</v>
@@ -36044,7 +36027,7 @@
       <c r="J774" s="2"/>
       <c r="K774" s="2"/>
     </row>
-    <row r="775" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="775" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A775" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Nate the Snake|NAME</v>
@@ -36073,7 +36056,7 @@
       <c r="J775" s="2"/>
       <c r="K775" s="2"/>
     </row>
-    <row r="776" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="776" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A776" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Nate the Snake|RUNE</v>
@@ -36102,7 +36085,7 @@
       <c r="J776" s="2"/>
       <c r="K776" s="2"/>
     </row>
-    <row r="777" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="777" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A777" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Nate the Snake|STON</v>
@@ -36131,7 +36114,7 @@
       <c r="J777" s="2"/>
       <c r="K777" s="2"/>
     </row>
-    <row r="778" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="778" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A778" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Ruskin|HEALTH</v>
@@ -36166,7 +36149,7 @@
       </c>
       <c r="K778" s="2"/>
     </row>
-    <row r="779" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="779" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A779" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Ruskin|HUMI</v>
@@ -36201,7 +36184,7 @@
       </c>
       <c r="K779" s="2"/>
     </row>
-    <row r="780" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="780" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A780" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Ruskin|JOB</v>
@@ -36236,7 +36219,7 @@
       </c>
       <c r="K780" s="2"/>
     </row>
-    <row r="781" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="781" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A781" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Ruskin|LOOK</v>
@@ -36271,7 +36254,7 @@
       </c>
       <c r="K781" s="2"/>
     </row>
-    <row r="782" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="782" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A782" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Ruskin|NAME</v>
@@ -36306,7 +36289,7 @@
       </c>
       <c r="K782" s="2"/>
     </row>
-    <row r="783" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="783" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A783" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Ruskin|RUNE</v>
@@ -36341,7 +36324,7 @@
       </c>
       <c r="K783" s="2"/>
     </row>
-    <row r="784" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="784" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A784" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Skullface|HEALTH</v>
@@ -36376,7 +36359,7 @@
       </c>
       <c r="K784" s="2"/>
     </row>
-    <row r="785" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="785" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A785" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Skullface|JOB</v>
@@ -36411,7 +36394,7 @@
       </c>
       <c r="K785" s="2"/>
     </row>
-    <row r="786" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="786" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A786" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Skullface|LOOK</v>
@@ -36446,7 +36429,7 @@
       </c>
       <c r="K786" s="2"/>
     </row>
-    <row r="787" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="787" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A787" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Skullface|NAME</v>
@@ -36481,7 +36464,7 @@
       </c>
       <c r="K787" s="2"/>
     </row>
-    <row r="788" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="788" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A788" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Slim|BONE</v>
@@ -36518,7 +36501,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="789" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="789" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A789" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Slim|HEALTH</v>
@@ -36555,7 +36538,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="790" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="790" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A790" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Slim|JOB</v>
@@ -36592,7 +36575,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="791" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="791" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A791" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Slim|LOOK</v>
@@ -36629,7 +36612,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="792" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="792" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A792" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Slim|NAME</v>
@@ -36666,7 +36649,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="793" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="793" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A793" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Slim|PRID</v>
@@ -36703,7 +36686,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="794" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="794" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A794" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Splot|HEALTH</v>
@@ -36738,7 +36721,7 @@
       </c>
       <c r="K794" s="2"/>
     </row>
-    <row r="795" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="795" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A795" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Splot|HUMB</v>
@@ -36773,7 +36756,7 @@
       </c>
       <c r="K795" s="2"/>
     </row>
-    <row r="796" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="796" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A796" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Splot|JOB</v>
@@ -36808,7 +36791,7 @@
       </c>
       <c r="K796" s="2"/>
     </row>
-    <row r="797" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="797" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A797" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Splot|LOOK</v>
@@ -36843,7 +36826,7 @@
       </c>
       <c r="K797" s="2"/>
     </row>
-    <row r="798" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="798" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A798" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Splot|NAME</v>
@@ -36878,7 +36861,7 @@
       </c>
       <c r="K798" s="2"/>
     </row>
-    <row r="799" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="799" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A799" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Splot|REGR</v>
@@ -36913,7 +36896,7 @@
       </c>
       <c r="K799" s="2"/>
     </row>
-    <row r="800" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="800" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A800" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Virtuebane|HEALTH</v>
@@ -36950,7 +36933,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="801" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="801" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A801" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Virtuebane|JOB</v>
@@ -36987,7 +36970,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="802" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="802" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A802" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Virtuebane|LOOK</v>
@@ -37024,7 +37007,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="803" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="803" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A803" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Virtuebane|MAGI</v>
@@ -37061,7 +37044,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="804" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="804" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A804" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Virtuebane|NAME</v>
@@ -37098,7 +37081,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="805" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="805" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A805" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Wierdrum|HAUN</v>
@@ -37127,7 +37110,7 @@
       <c r="J805" s="2"/>
       <c r="K805" s="2"/>
     </row>
-    <row r="806" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="806" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A806" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Wierdrum|HEALTH</v>
@@ -37156,7 +37139,7 @@
       <c r="J806" s="2"/>
       <c r="K806" s="2"/>
     </row>
-    <row r="807" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="807" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A807" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Wierdrum|JOB</v>
@@ -37185,7 +37168,7 @@
       <c r="J807" s="2"/>
       <c r="K807" s="2"/>
     </row>
-    <row r="808" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="808" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A808" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Wierdrum|LOOK</v>
@@ -37214,7 +37197,7 @@
       <c r="J808" s="2"/>
       <c r="K808" s="2"/>
     </row>
-    <row r="809" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="809" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A809" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Wierdrum|NAME</v>
@@ -37243,7 +37226,7 @@
       <c r="J809" s="2"/>
       <c r="K809" s="2"/>
     </row>
-    <row r="810" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="810" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A810" t="str">
         <f t="shared" si="12"/>
         <v>Magincia|Wierdrum|SHRI</v>
@@ -37272,7 +37255,7 @@
       <c r="J810" s="2"/>
       <c r="K810" s="2"/>
     </row>
-    <row r="811" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="811" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A811" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Alex|FLOW</v>
@@ -37307,7 +37290,7 @@
       </c>
       <c r="K811" s="2"/>
     </row>
-    <row r="812" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="812" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A812" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Alex|HEALTH</v>
@@ -37342,7 +37325,7 @@
       </c>
       <c r="K812" s="2"/>
     </row>
-    <row r="813" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="813" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A813" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Alex|JOB</v>
@@ -37377,7 +37360,7 @@
       </c>
       <c r="K813" s="2"/>
     </row>
-    <row r="814" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="814" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A814" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Alex|KIND</v>
@@ -37412,7 +37395,7 @@
       </c>
       <c r="K814" s="2"/>
     </row>
-    <row r="815" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="815" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A815" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Alex|LOOK</v>
@@ -37430,7 +37413,7 @@
         <v>16</v>
       </c>
       <c r="F815" s="2" t="s">
-        <v>2606</v>
+        <v>2605</v>
       </c>
       <c r="G815" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B815&amp;"|"&amp;C815&amp;"|"&amp;D815&amp;"|"&amp;E815,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -37447,7 +37430,7 @@
       </c>
       <c r="K815" s="2"/>
     </row>
-    <row r="816" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="816" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A816" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Alex|NAME</v>
@@ -37692,7 +37675,7 @@
       </c>
       <c r="K822" s="2"/>
     </row>
-    <row r="823" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="823" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A823" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Azure|HEALTH</v>
@@ -37727,7 +37710,7 @@
       </c>
       <c r="K823" s="2"/>
     </row>
-    <row r="824" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="824" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A824" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Azure|JOB</v>
@@ -37762,7 +37745,7 @@
       </c>
       <c r="K824" s="2"/>
     </row>
-    <row r="825" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="825" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A825" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Azure|LOOK</v>
@@ -37797,7 +37780,7 @@
       </c>
       <c r="K825" s="2"/>
     </row>
-    <row r="826" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="826" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A826" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Azure|NAME</v>
@@ -37832,7 +37815,7 @@
       </c>
       <c r="K826" s="2"/>
     </row>
-    <row r="827" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="827" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A827" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Azure|RUNE</v>
@@ -37867,7 +37850,7 @@
       </c>
       <c r="K827" s="2"/>
     </row>
-    <row r="828" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="828" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A828" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Azure|SACR</v>
@@ -37902,7 +37885,7 @@
       </c>
       <c r="K828" s="2"/>
     </row>
-    <row r="829" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="829" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A829" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Bob the Beggar|HEALTH</v>
@@ -37937,7 +37920,7 @@
       </c>
       <c r="K829" s="2"/>
     </row>
-    <row r="830" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="830" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A830" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Bob the Beggar|HELP</v>
@@ -37972,7 +37955,7 @@
       </c>
       <c r="K830" s="2"/>
     </row>
-    <row r="831" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="831" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A831" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Bob the Beggar|JOB</v>
@@ -38007,7 +37990,7 @@
       </c>
       <c r="K831" s="2"/>
     </row>
-    <row r="832" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="832" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A832" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Bob the Beggar|LOOK</v>
@@ -38042,7 +38025,7 @@
       </c>
       <c r="K832" s="2"/>
     </row>
-    <row r="833" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="833" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A833" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Bob the Beggar|NAME</v>
@@ -38077,7 +38060,7 @@
       </c>
       <c r="K833" s="2"/>
     </row>
-    <row r="834" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="834" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A834" t="str">
         <f t="shared" si="12"/>
         <v>Minoc|Bob the Beggar|SICK</v>
@@ -38112,7 +38095,7 @@
       </c>
       <c r="K834" s="2"/>
     </row>
-    <row r="835" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="835" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A835" t="str">
         <f t="shared" ref="A835:A898" si="13">C835&amp;"|"&amp;D835&amp;"|"&amp;E835</f>
         <v>Minoc|Damon|HEALTH</v>
@@ -38147,7 +38130,7 @@
       </c>
       <c r="K835" s="2"/>
     </row>
-    <row r="836" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="836" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A836" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Damon|JOB</v>
@@ -38182,7 +38165,7 @@
       </c>
       <c r="K836" s="2"/>
     </row>
-    <row r="837" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="837" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A837" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Damon|LOOK</v>
@@ -38217,7 +38200,7 @@
       </c>
       <c r="K837" s="2"/>
     </row>
-    <row r="838" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="838" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A838" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Damon|MANT</v>
@@ -38252,7 +38235,7 @@
       </c>
       <c r="K838" s="2"/>
     </row>
-    <row r="839" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="839" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A839" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Damon|NAME</v>
@@ -38287,7 +38270,7 @@
       </c>
       <c r="K839" s="2"/>
     </row>
-    <row r="840" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="840" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A840" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Damon|THIN</v>
@@ -38532,7 +38515,7 @@
       </c>
       <c r="K846" s="2"/>
     </row>
-    <row r="847" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="847" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A847" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Gimble|CONS</v>
@@ -38567,7 +38550,7 @@
       </c>
       <c r="K847" s="2"/>
     </row>
-    <row r="848" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="848" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A848" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Gimble|DIE</v>
@@ -38602,7 +38585,7 @@
       </c>
       <c r="K848" s="2"/>
     </row>
-    <row r="849" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="849" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A849" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Gimble|HEALTH</v>
@@ -38637,7 +38620,7 @@
       </c>
       <c r="K849" s="2"/>
     </row>
-    <row r="850" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="850" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A850" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Gimble|JOB</v>
@@ -38672,7 +38655,7 @@
       </c>
       <c r="K850" s="2"/>
     </row>
-    <row r="851" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="851" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A851" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Gimble|LOOK</v>
@@ -38707,7 +38690,7 @@
       </c>
       <c r="K851" s="2"/>
     </row>
-    <row r="852" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="852" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A852" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Gimble|NAME</v>
@@ -38742,7 +38725,7 @@
       </c>
       <c r="K852" s="2"/>
     </row>
-    <row r="853" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="853" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A853" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Jude|HEALTH</v>
@@ -38777,7 +38760,7 @@
       </c>
       <c r="K853" s="2"/>
     </row>
-    <row r="854" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="854" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A854" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Jude|JOB</v>
@@ -38812,7 +38795,7 @@
       </c>
       <c r="K854" s="2"/>
     </row>
-    <row r="855" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="855" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A855" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Jude|LOOK</v>
@@ -38847,7 +38830,7 @@
       </c>
       <c r="K855" s="2"/>
     </row>
-    <row r="856" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="856" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A856" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Jude|NAME</v>
@@ -38882,7 +38865,7 @@
       </c>
       <c r="K856" s="2"/>
     </row>
-    <row r="857" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="857" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A857" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Jude|REDE</v>
@@ -38917,7 +38900,7 @@
       </c>
       <c r="K857" s="2"/>
     </row>
-    <row r="858" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="858" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A858" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Jude|SKUL</v>
@@ -38952,7 +38935,7 @@
       </c>
       <c r="K858" s="2"/>
     </row>
-    <row r="859" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="859" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A859" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Julia|CARE</v>
@@ -38987,7 +38970,7 @@
       </c>
       <c r="K859" s="2"/>
     </row>
-    <row r="860" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="860" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A860" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Julia|HEALTH</v>
@@ -39022,7 +39005,7 @@
       </c>
       <c r="K860" s="2"/>
     </row>
-    <row r="861" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="861" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A861" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Julia|JOB</v>
@@ -39057,7 +39040,7 @@
       </c>
       <c r="K861" s="2"/>
     </row>
-    <row r="862" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="862" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A862" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Julia|LOOK</v>
@@ -39092,7 +39075,7 @@
       </c>
       <c r="K862" s="2"/>
     </row>
-    <row r="863" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="863" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A863" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Julia|NAME</v>
@@ -39127,7 +39110,7 @@
       </c>
       <c r="K863" s="2"/>
     </row>
-    <row r="864" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="864" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A864" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Julia|POOR</v>
@@ -39372,7 +39355,7 @@
       </c>
       <c r="K870" s="2"/>
     </row>
-    <row r="871" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="871" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A871" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Merida|HEALTH</v>
@@ -39407,7 +39390,7 @@
       </c>
       <c r="K871" s="2"/>
     </row>
-    <row r="872" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="872" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A872" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Merida|JOB</v>
@@ -39442,7 +39425,7 @@
       </c>
       <c r="K872" s="2"/>
     </row>
-    <row r="873" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="873" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A873" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Merida|LOOK</v>
@@ -39477,7 +39460,7 @@
       </c>
       <c r="K873" s="2"/>
     </row>
-    <row r="874" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="874" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A874" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Merida|MANT</v>
@@ -39512,7 +39495,7 @@
       </c>
       <c r="K874" s="2"/>
     </row>
-    <row r="875" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="875" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A875" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Merida|NAME</v>
@@ -39547,7 +39530,7 @@
       </c>
       <c r="K875" s="2"/>
     </row>
-    <row r="876" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="876" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A876" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Merida|SHRI</v>
@@ -39582,7 +39565,7 @@
       </c>
       <c r="K876" s="2"/>
     </row>
-    <row r="877" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="877" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A877" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mike Ward|HEALTH</v>
@@ -39617,7 +39600,7 @@
       </c>
       <c r="K877" s="2"/>
     </row>
-    <row r="878" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="878" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A878" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mike Ward|JOB</v>
@@ -39652,7 +39635,7 @@
       </c>
       <c r="K878" s="2"/>
     </row>
-    <row r="879" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="879" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A879" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mike Ward|LOOK</v>
@@ -39687,7 +39670,7 @@
       </c>
       <c r="K879" s="2"/>
     </row>
-    <row r="880" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="880" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A880" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mike Ward|NAME</v>
@@ -39722,7 +39705,7 @@
       </c>
       <c r="K880" s="2"/>
     </row>
-    <row r="881" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="881" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A881" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mike Ward|ROOM</v>
@@ -39757,7 +39740,7 @@
       </c>
       <c r="K881" s="2"/>
     </row>
-    <row r="882" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="882" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A882" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mike Ward|SKAR</v>
@@ -39792,7 +39775,7 @@
       </c>
       <c r="K882" s="2"/>
     </row>
-    <row r="883" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="883" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A883" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mischief|HEALTH</v>
@@ -39820,14 +39803,14 @@
         <v>1194</v>
       </c>
       <c r="I883" s="41" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="J883" s="2" t="s">
         <v>1195</v>
       </c>
       <c r="K883" s="2"/>
     </row>
-    <row r="884" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="884" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A884" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mischief|JOB</v>
@@ -39855,14 +39838,14 @@
         <v>1194</v>
       </c>
       <c r="I884" s="41" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="J884" s="2" t="s">
         <v>1195</v>
       </c>
       <c r="K884" s="2"/>
     </row>
-    <row r="885" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="885" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A885" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mischief|LOOK</v>
@@ -39890,14 +39873,14 @@
         <v>1194</v>
       </c>
       <c r="I885" s="41" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="J885" s="2" t="s">
         <v>1195</v>
       </c>
       <c r="K885" s="2"/>
     </row>
-    <row r="886" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="886" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A886" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mischief|NAME</v>
@@ -39925,14 +39908,14 @@
         <v>1194</v>
       </c>
       <c r="I886" s="41" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="J886" s="2" t="s">
         <v>1195</v>
       </c>
       <c r="K886" s="2"/>
     </row>
-    <row r="887" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="887" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A887" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mischief|RUNE</v>
@@ -39960,14 +39943,14 @@
         <v>1194</v>
       </c>
       <c r="I887" s="41" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="J887" s="2" t="s">
         <v>1195</v>
       </c>
       <c r="K887" s="2"/>
     </row>
-    <row r="888" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="888" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A888" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Mischief|FORGE</v>
@@ -39982,10 +39965,10 @@
         <v>1193</v>
       </c>
       <c r="E888" s="2" t="s">
+        <v>2600</v>
+      </c>
+      <c r="F888" s="3" t="s">
         <v>2601</v>
-      </c>
-      <c r="F888" s="3" t="s">
-        <v>2602</v>
       </c>
       <c r="G888" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B888&amp;"|"&amp;C888&amp;"|"&amp;D888&amp;"|"&amp;E888,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -39995,14 +39978,14 @@
         <v>1194</v>
       </c>
       <c r="I888" s="41" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="J888" s="2" t="s">
         <v>1195</v>
       </c>
       <c r="K888" s="2"/>
     </row>
-    <row r="889" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="889" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A889" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Shentis|HEALTH</v>
@@ -40037,7 +40020,7 @@
       </c>
       <c r="K889" s="2"/>
     </row>
-    <row r="890" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="890" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A890" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Shentis|JOB</v>
@@ -40072,7 +40055,7 @@
       </c>
       <c r="K890" s="2"/>
     </row>
-    <row r="891" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="891" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A891" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Shentis|LOOK</v>
@@ -40107,7 +40090,7 @@
       </c>
       <c r="K891" s="2"/>
     </row>
-    <row r="892" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="892" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A892" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Shentis|NAME</v>
@@ -40142,7 +40125,7 @@
       </c>
       <c r="K892" s="2"/>
     </row>
-    <row r="893" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="893" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A893" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Shentis|SACR</v>
@@ -40177,7 +40160,7 @@
       </c>
       <c r="K893" s="2"/>
     </row>
-    <row r="894" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="894" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A894" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Shentis|VIRT</v>
@@ -40212,7 +40195,7 @@
       </c>
       <c r="K894" s="2"/>
     </row>
-    <row r="895" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="895" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A895" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Singsong|HEALTH</v>
@@ -40241,7 +40224,7 @@
       <c r="J895" s="2"/>
       <c r="K895" s="2"/>
     </row>
-    <row r="896" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="896" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A896" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Singsong|JOB</v>
@@ -40270,7 +40253,7 @@
       <c r="J896" s="2"/>
       <c r="K896" s="2"/>
     </row>
-    <row r="897" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="897" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A897" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Singsong|LOOK</v>
@@ -40299,7 +40282,7 @@
       <c r="J897" s="2"/>
       <c r="K897" s="2"/>
     </row>
-    <row r="898" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="898" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A898" t="str">
         <f t="shared" si="13"/>
         <v>Minoc|Singsong|NAME</v>
@@ -40328,7 +40311,7 @@
       <c r="J898" s="2"/>
       <c r="K898" s="2"/>
     </row>
-    <row r="899" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="899" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A899" t="str">
         <f t="shared" ref="A899:A962" si="14">C899&amp;"|"&amp;D899&amp;"|"&amp;E899</f>
         <v>Minoc|Singsong|SING</v>
@@ -40357,7 +40340,7 @@
       <c r="J899" s="2"/>
       <c r="K899" s="2"/>
     </row>
-    <row r="900" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="900" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A900" t="str">
         <f t="shared" si="14"/>
         <v>Minoc|Singsong|SONG</v>
@@ -40386,7 +40369,7 @@
       <c r="J900" s="2"/>
       <c r="K900" s="2"/>
     </row>
-    <row r="901" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="901" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A901" t="str">
         <f t="shared" si="14"/>
         <v>Minoc|Zircon|HEALTH</v>
@@ -40421,7 +40404,7 @@
       </c>
       <c r="K901" s="2"/>
     </row>
-    <row r="902" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="902" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A902" t="str">
         <f t="shared" si="14"/>
         <v>Minoc|Zircon|JOB</v>
@@ -40456,7 +40439,7 @@
       </c>
       <c r="K902" s="2"/>
     </row>
-    <row r="903" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="903" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A903" t="str">
         <f t="shared" si="14"/>
         <v>Minoc|Zircon|LOOK</v>
@@ -40491,7 +40474,7 @@
       </c>
       <c r="K903" s="2"/>
     </row>
-    <row r="904" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="904" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A904" t="str">
         <f t="shared" si="14"/>
         <v>Minoc|Zircon|MYST</v>
@@ -40526,7 +40509,7 @@
       </c>
       <c r="K904" s="2"/>
     </row>
-    <row r="905" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="905" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A905" t="str">
         <f t="shared" si="14"/>
         <v>Minoc|Zircon|NAME</v>
@@ -40561,7 +40544,7 @@
       </c>
       <c r="K905" s="2"/>
     </row>
-    <row r="906" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="906" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A906" t="str">
         <f t="shared" si="14"/>
         <v>Minoc|Zircon|WEAP</v>
@@ -50542,7 +50525,7 @@
       </c>
       <c r="K1191" s="2"/>
     </row>
-    <row r="1192" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1192" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1192" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Ambule|BEG</v>
@@ -50577,7 +50560,7 @@
       </c>
       <c r="K1192" s="2"/>
     </row>
-    <row r="1193" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1193" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1193" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Ambule|HEALTH</v>
@@ -50612,7 +50595,7 @@
       </c>
       <c r="K1193" s="2"/>
     </row>
-    <row r="1194" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1194" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1194" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Ambule|JOB</v>
@@ -50647,7 +50630,7 @@
       </c>
       <c r="K1194" s="2"/>
     </row>
-    <row r="1195" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1195" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1195" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Ambule|LOOK</v>
@@ -50682,7 +50665,7 @@
       </c>
       <c r="K1195" s="2"/>
     </row>
-    <row r="1196" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1196" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1196" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Ambule|MANT</v>
@@ -50700,7 +50683,7 @@
         <v>742</v>
       </c>
       <c r="F1196" s="41" t="s">
-        <v>2597</v>
+        <v>2596</v>
       </c>
       <c r="G1196" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B1196&amp;"|"&amp;C1196&amp;"|"&amp;D1196&amp;"|"&amp;E1196,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -50717,7 +50700,7 @@
       </c>
       <c r="K1196" s="2"/>
     </row>
-    <row r="1197" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1197" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1197" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Ambule|NAME</v>
@@ -50962,7 +50945,7 @@
       </c>
       <c r="K1203" s="2"/>
     </row>
-    <row r="1204" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1204" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1204" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Barren|HEALTH</v>
@@ -50991,7 +50974,7 @@
       <c r="J1204" s="2"/>
       <c r="K1204" s="2"/>
     </row>
-    <row r="1205" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1205" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1205" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Barren|JOB</v>
@@ -51009,7 +50992,7 @@
         <v>18</v>
       </c>
       <c r="F1205" s="2" t="s">
-        <v>2598</v>
+        <v>2597</v>
       </c>
       <c r="G1205" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B1205&amp;"|"&amp;C1205&amp;"|"&amp;D1205&amp;"|"&amp;E1205,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -51020,7 +51003,7 @@
       <c r="J1205" s="2"/>
       <c r="K1205" s="2"/>
     </row>
-    <row r="1206" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1206" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1206" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Barren|LOOK</v>
@@ -51038,7 +51021,7 @@
         <v>16</v>
       </c>
       <c r="F1206" s="41" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="G1206" s="8" t="str">
         <f>IF(ISNA(VLOOKUP(B1206&amp;"|"&amp;C1206&amp;"|"&amp;D1206&amp;"|"&amp;E1206,QuestionTriggers!A:F,6,FALSE)),"","---&gt;")</f>
@@ -51049,7 +51032,7 @@
       <c r="J1206" s="2"/>
       <c r="K1206" s="2"/>
     </row>
-    <row r="1207" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1207" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1207" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Barren|MANT</v>
@@ -51078,7 +51061,7 @@
       <c r="J1207" s="2"/>
       <c r="K1207" s="2"/>
     </row>
-    <row r="1208" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1208" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1208" t="str">
         <f t="shared" si="18"/>
         <v>Skara Brae|Barren|NAME</v>
@@ -51682,7 +51665,7 @@
       </c>
       <c r="K1225" s="2"/>
     </row>
-    <row r="1226" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1226" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1226" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Emerson|HEALTH</v>
@@ -51717,7 +51700,7 @@
       </c>
       <c r="K1226" s="2"/>
     </row>
-    <row r="1227" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1227" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1227" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Emerson|JOB</v>
@@ -51752,7 +51735,7 @@
       </c>
       <c r="K1227" s="2"/>
     </row>
-    <row r="1228" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1228" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1228" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Emerson|LOOK</v>
@@ -51787,7 +51770,7 @@
       </c>
       <c r="K1228" s="2"/>
     </row>
-    <row r="1229" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1229" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1229" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Emerson|NAME</v>
@@ -51822,7 +51805,7 @@
       </c>
       <c r="K1229" s="2"/>
     </row>
-    <row r="1230" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1230" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1230" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Emerson|SPIR</v>
@@ -51857,7 +51840,7 @@
       </c>
       <c r="K1230" s="2"/>
     </row>
-    <row r="1231" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1231" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1231" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Emerson|WOUN</v>
@@ -51892,7 +51875,7 @@
       </c>
       <c r="K1231" s="2"/>
     </row>
-    <row r="1232" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1232" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A1232" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Granted|FOOD</v>
@@ -51927,7 +51910,7 @@
       </c>
       <c r="K1232" s="2"/>
     </row>
-    <row r="1233" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1233" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A1233" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Granted|HEALTH</v>
@@ -51962,7 +51945,7 @@
       </c>
       <c r="K1233" s="2"/>
     </row>
-    <row r="1234" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1234" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A1234" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Granted|JOB</v>
@@ -51997,7 +51980,7 @@
       </c>
       <c r="K1234" s="2"/>
     </row>
-    <row r="1235" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1235" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A1235" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Granted|LOOK</v>
@@ -52032,7 +52015,7 @@
       </c>
       <c r="K1235" s="2"/>
     </row>
-    <row r="1236" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1236" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A1236" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Granted|MONE</v>
@@ -52067,7 +52050,7 @@
       </c>
       <c r="K1236" s="2"/>
     </row>
-    <row r="1237" spans="1:11" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1237" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A1237" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Granted|NAME</v>
@@ -52102,7 +52085,7 @@
       </c>
       <c r="K1237" s="2"/>
     </row>
-    <row r="1238" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1238" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1238" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Isaac|HAUN</v>
@@ -52137,7 +52120,7 @@
       </c>
       <c r="K1238" s="2"/>
     </row>
-    <row r="1239" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1239" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1239" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Isaac|HEALTH</v>
@@ -52172,7 +52155,7 @@
       </c>
       <c r="K1239" s="2"/>
     </row>
-    <row r="1240" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1240" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1240" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Isaac|JOB</v>
@@ -52207,7 +52190,7 @@
       </c>
       <c r="K1240" s="2"/>
     </row>
-    <row r="1241" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1241" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1241" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Isaac|LOOK</v>
@@ -52242,7 +52225,7 @@
       </c>
       <c r="K1241" s="2"/>
     </row>
-    <row r="1242" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1242" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1242" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Isaac|NAME</v>
@@ -52277,7 +52260,7 @@
       </c>
       <c r="K1242" s="2"/>
     </row>
-    <row r="1243" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1243" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1243" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Isaac|STON</v>
@@ -52732,7 +52715,7 @@
       </c>
       <c r="K1255" s="2"/>
     </row>
-    <row r="1256" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1256" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1256" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Presto|HEALTH</v>
@@ -52767,7 +52750,7 @@
       </c>
       <c r="K1256" s="2"/>
     </row>
-    <row r="1257" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1257" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1257" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Presto|JOB</v>
@@ -52802,7 +52785,7 @@
       </c>
       <c r="K1257" s="2"/>
     </row>
-    <row r="1258" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1258" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1258" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Presto|LOOK</v>
@@ -52837,7 +52820,7 @@
       </c>
       <c r="K1258" s="2"/>
     </row>
-    <row r="1259" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1259" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1259" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Presto|NAME</v>
@@ -52872,7 +52855,7 @@
       </c>
       <c r="K1259" s="2"/>
     </row>
-    <row r="1260" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1260" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1260" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Presto|NIGH</v>
@@ -52907,7 +52890,7 @@
       </c>
       <c r="K1260" s="2"/>
     </row>
-    <row r="1261" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1261" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1261" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Presto|SPEL</v>
@@ -52942,7 +52925,7 @@
       </c>
       <c r="K1261" s="2"/>
     </row>
-    <row r="1262" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1262" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1262" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Romasco|HEALTH</v>
@@ -52977,7 +52960,7 @@
       </c>
       <c r="K1262" s="2"/>
     </row>
-    <row r="1263" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1263" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1263" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Romasco|JOB</v>
@@ -53012,7 +52995,7 @@
       </c>
       <c r="K1263" s="2"/>
     </row>
-    <row r="1264" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1264" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1264" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Romasco|LOOK</v>
@@ -53047,7 +53030,7 @@
       </c>
       <c r="K1264" s="2"/>
     </row>
-    <row r="1265" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1265" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1265" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Romasco|NAME</v>
@@ -53082,7 +53065,7 @@
       </c>
       <c r="K1265" s="2"/>
     </row>
-    <row r="1266" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1266" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1266" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Romasco|TEAC</v>
@@ -53117,7 +53100,7 @@
       </c>
       <c r="K1266" s="2"/>
     </row>
-    <row r="1267" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1267" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1267" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Romasco|WORD</v>
@@ -53152,7 +53135,7 @@
       </c>
       <c r="K1267" s="2"/>
     </row>
-    <row r="1268" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1268" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1268" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Santayana|HEALTH</v>
@@ -53187,7 +53170,7 @@
       </c>
       <c r="K1268" s="2"/>
     </row>
-    <row r="1269" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1269" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1269" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Santayana|JOB</v>
@@ -53222,7 +53205,7 @@
       </c>
       <c r="K1269" s="2"/>
     </row>
-    <row r="1270" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1270" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1270" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Santayana|LIGH</v>
@@ -53257,7 +53240,7 @@
       </c>
       <c r="K1270" s="2"/>
     </row>
-    <row r="1271" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1271" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1271" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Santayana|LOOK</v>
@@ -53292,7 +53275,7 @@
       </c>
       <c r="K1271" s="2"/>
     </row>
-    <row r="1272" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1272" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1272" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Santayana|NAME</v>
@@ -53327,7 +53310,7 @@
       </c>
       <c r="K1272" s="2"/>
     </row>
-    <row r="1273" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1273" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1273" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Santayana|PHIL</v>
@@ -53362,7 +53345,7 @@
       </c>
       <c r="K1273" s="2"/>
     </row>
-    <row r="1274" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1274" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1274" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Shamino|HEALTH</v>
@@ -53397,7 +53380,7 @@
       </c>
       <c r="K1274" s="2"/>
     </row>
-    <row r="1275" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1275" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1275" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Shamino|JOB</v>
@@ -53432,7 +53415,7 @@
       </c>
       <c r="K1275" s="2"/>
     </row>
-    <row r="1276" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1276" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1276" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Shamino|LIGH</v>
@@ -53467,7 +53450,7 @@
       </c>
       <c r="K1276" s="2"/>
     </row>
-    <row r="1277" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1277" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1277" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Shamino|LOOK</v>
@@ -53502,7 +53485,7 @@
       </c>
       <c r="K1277" s="2"/>
     </row>
-    <row r="1278" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1278" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1278" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Shamino|NAME</v>
@@ -53537,7 +53520,7 @@
       </c>
       <c r="K1278" s="2"/>
     </row>
-    <row r="1279" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1279" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1279" t="str">
         <f t="shared" si="19"/>
         <v>Skara Brae|Shamino|TRUT</v>
@@ -60387,7 +60370,7 @@
       </c>
       <c r="K1476" s="2"/>
     </row>
-    <row r="1477" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1477" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1477" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Beggar|FELO</v>
@@ -60422,7 +60405,7 @@
       </c>
       <c r="K1477" s="2"/>
     </row>
-    <row r="1478" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1478" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1478" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Beggar|HEALTH</v>
@@ -60457,7 +60440,7 @@
       </c>
       <c r="K1478" s="2"/>
     </row>
-    <row r="1479" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1479" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1479" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Beggar|JOB</v>
@@ -60492,7 +60475,7 @@
       </c>
       <c r="K1479" s="2"/>
     </row>
-    <row r="1480" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1480" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1480" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Beggar|LOOK</v>
@@ -60527,7 +60510,7 @@
       </c>
       <c r="K1480" s="2"/>
     </row>
-    <row r="1481" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1481" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1481" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Beggar|NAME</v>
@@ -60562,7 +60545,7 @@
       </c>
       <c r="K1481" s="2"/>
     </row>
-    <row r="1482" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1482" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1482" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Beggar|I have sinned.</v>
@@ -60597,7 +60580,7 @@
       </c>
       <c r="K1482" s="2"/>
     </row>
-    <row r="1483" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1483" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1483" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Calumny|HEALTH</v>
@@ -60632,7 +60615,7 @@
       </c>
       <c r="K1483" s="2"/>
     </row>
-    <row r="1484" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1484" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1484" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Calumny|JOB</v>
@@ -60667,7 +60650,7 @@
       </c>
       <c r="K1484" s="2"/>
     </row>
-    <row r="1485" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1485" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1485" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Calumny|LOOK</v>
@@ -60702,7 +60685,7 @@
       </c>
       <c r="K1485" s="2"/>
     </row>
-    <row r="1486" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1486" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1486" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Calumny|MAND</v>
@@ -60737,7 +60720,7 @@
       </c>
       <c r="K1486" s="2"/>
     </row>
-    <row r="1487" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1487" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1487" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Calumny|NAME</v>
@@ -60772,7 +60755,7 @@
       </c>
       <c r="K1487" s="2"/>
     </row>
-    <row r="1488" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1488" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1488" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Calumny|SPEL</v>
@@ -60807,7 +60790,7 @@
       </c>
       <c r="K1488" s="2"/>
     </row>
-    <row r="1489" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1489" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1489" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Court Guard|COUR</v>
@@ -60842,7 +60825,7 @@
       </c>
       <c r="K1489" s="2"/>
     </row>
-    <row r="1490" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1490" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1490" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Court Guard|HEALTH</v>
@@ -60877,7 +60860,7 @@
       </c>
       <c r="K1490" s="2"/>
     </row>
-    <row r="1491" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1491" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1491" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Court Guard|JOB</v>
@@ -60912,7 +60895,7 @@
       </c>
       <c r="K1491" s="2"/>
     </row>
-    <row r="1492" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1492" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1492" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Court Guard|JUST</v>
@@ -60947,7 +60930,7 @@
       </c>
       <c r="K1492" s="2"/>
     </row>
-    <row r="1493" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1493" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1493" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Court Guard|LOOK</v>
@@ -60982,7 +60965,7 @@
       </c>
       <c r="K1493" s="2"/>
     </row>
-    <row r="1494" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1494" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1494" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Court Guard|NAME</v>
@@ -61017,7 +61000,7 @@
       </c>
       <c r="K1494" s="2"/>
     </row>
-    <row r="1495" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1495" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1495" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Druid|HEALTH</v>
@@ -61052,7 +61035,7 @@
       </c>
       <c r="K1495" s="2"/>
     </row>
-    <row r="1496" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1496" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1496" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Druid|JOB</v>
@@ -61087,7 +61070,7 @@
       </c>
       <c r="K1496" s="2"/>
     </row>
-    <row r="1497" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1497" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1497" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Druid|JUST</v>
@@ -61122,7 +61105,7 @@
       </c>
       <c r="K1497" s="2"/>
     </row>
-    <row r="1498" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1498" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1498" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Druid|LOOK</v>
@@ -61157,7 +61140,7 @@
       </c>
       <c r="K1498" s="2"/>
     </row>
-    <row r="1499" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1499" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1499" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Druid|NAME</v>
@@ -61192,7 +61175,7 @@
       </c>
       <c r="K1499" s="2"/>
     </row>
-    <row r="1500" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1500" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1500" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Druid|SHRI</v>
@@ -61227,7 +61210,7 @@
       </c>
       <c r="K1500" s="2"/>
     </row>
-    <row r="1501" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1501" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1501" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Dwp|HEALTH</v>
@@ -61262,7 +61245,7 @@
       </c>
       <c r="K1501" s="2"/>
     </row>
-    <row r="1502" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1502" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1502" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Dwp|JOB</v>
@@ -61297,7 +61280,7 @@
       </c>
       <c r="K1502" s="2"/>
     </row>
-    <row r="1503" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1503" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1503" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Dwp|JUST</v>
@@ -61332,7 +61315,7 @@
       </c>
       <c r="K1503" s="2"/>
     </row>
-    <row r="1504" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1504" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1504" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Dwp|LOOK</v>
@@ -61367,7 +61350,7 @@
       </c>
       <c r="K1504" s="2"/>
     </row>
-    <row r="1505" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1505" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1505" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Dwp|NAME</v>
@@ -61402,7 +61385,7 @@
       </c>
       <c r="K1505" s="2"/>
     </row>
-    <row r="1506" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1506" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1506" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Dwp|YEW</v>
@@ -61694,7 +61677,7 @@
       </c>
       <c r="K1513" s="2"/>
     </row>
-    <row r="1514" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1514" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1514" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Frida|HEALTH</v>
@@ -61729,7 +61712,7 @@
       </c>
       <c r="K1514" s="2"/>
     </row>
-    <row r="1515" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1515" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1515" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Frida|JOB</v>
@@ -61799,7 +61782,7 @@
       </c>
       <c r="K1516" s="2"/>
     </row>
-    <row r="1517" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1517" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1517" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Frida|LOOK</v>
@@ -61834,7 +61817,7 @@
       </c>
       <c r="K1517" s="2"/>
     </row>
-    <row r="1518" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1518" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1518" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Frida|NAME</v>
@@ -61869,7 +61852,7 @@
       </c>
       <c r="K1518" s="2"/>
     </row>
-    <row r="1519" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1519" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1519" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Guard|HEALTH</v>
@@ -61906,7 +61889,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1520" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1520" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1520" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Guard|JOB</v>
@@ -61943,7 +61926,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1521" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1521" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1521" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Guard|JUST</v>
@@ -61980,7 +61963,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1522" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1522" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1522" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Guard|LOOK</v>
@@ -62017,7 +62000,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1523" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1523" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1523" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Guard|NAME</v>
@@ -62054,7 +62037,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1524" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1524" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1524" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Guard|PEAC</v>
@@ -62091,7 +62074,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1525" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1525" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1525" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jaana|HEALTH</v>
@@ -62126,7 +62109,7 @@
       </c>
       <c r="K1525" s="2"/>
     </row>
-    <row r="1526" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1526" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1526" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jaana|JOB</v>
@@ -62161,7 +62144,7 @@
       </c>
       <c r="K1526" s="2"/>
     </row>
-    <row r="1527" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1527" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1527" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jaana|JUST</v>
@@ -62196,7 +62179,7 @@
       </c>
       <c r="K1527" s="2"/>
     </row>
-    <row r="1528" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1528" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1528" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jaana|LOOK</v>
@@ -62231,7 +62214,7 @@
       </c>
       <c r="K1528" s="2"/>
     </row>
-    <row r="1529" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1529" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1529" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jaana|NAME</v>
@@ -62266,7 +62249,7 @@
       </c>
       <c r="K1529" s="2"/>
     </row>
-    <row r="1530" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1530" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1530" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jaana|UNDE</v>
@@ -62301,7 +62284,7 @@
       </c>
       <c r="K1530" s="2"/>
     </row>
-    <row r="1531" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1531" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1531" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jail Guard|FELO</v>
@@ -62336,7 +62319,7 @@
       </c>
       <c r="K1531" s="2"/>
     </row>
-    <row r="1532" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1532" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1532" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jail Guard|HEALTH</v>
@@ -62371,7 +62354,7 @@
       </c>
       <c r="K1532" s="2"/>
     </row>
-    <row r="1533" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1533" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1533" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jail Guard|JOB</v>
@@ -62406,7 +62389,7 @@
       </c>
       <c r="K1533" s="2"/>
     </row>
-    <row r="1534" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1534" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1534" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jail Guard|LOOK</v>
@@ -62441,7 +62424,7 @@
       </c>
       <c r="K1534" s="2"/>
     </row>
-    <row r="1535" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1535" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1535" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jail Guard|MISD</v>
@@ -62476,7 +62459,7 @@
       </c>
       <c r="K1535" s="2"/>
     </row>
-    <row r="1536" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1536" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1536" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Jail Guard|NAME</v>
@@ -62511,7 +62494,7 @@
       </c>
       <c r="K1536" s="2"/>
     </row>
-    <row r="1537" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1537" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1537" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Pinrod|COUN</v>
@@ -62546,7 +62529,7 @@
       </c>
       <c r="K1537" s="2"/>
     </row>
-    <row r="1538" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1538" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1538" t="str">
         <f t="shared" si="23"/>
         <v>Yew|Pinrod|HEALTH</v>
@@ -62581,7 +62564,7 @@
       </c>
       <c r="K1538" s="2"/>
     </row>
-    <row r="1539" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1539" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1539" t="str">
         <f t="shared" ref="A1539:A1602" si="24">C1539&amp;"|"&amp;D1539&amp;"|"&amp;E1539</f>
         <v>Yew|Pinrod|JOB</v>
@@ -62616,7 +62599,7 @@
       </c>
       <c r="K1539" s="2"/>
     </row>
-    <row r="1540" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1540" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1540" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Pinrod|JUST</v>
@@ -62651,7 +62634,7 @@
       </c>
       <c r="K1540" s="2"/>
     </row>
-    <row r="1541" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1541" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1541" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Pinrod|LOOK</v>
@@ -62686,7 +62669,7 @@
       </c>
       <c r="K1541" s="2"/>
     </row>
-    <row r="1542" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1542" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1542" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Pinrod|NAME</v>
@@ -62721,7 +62704,7 @@
       </c>
       <c r="K1542" s="2"/>
     </row>
-    <row r="1543" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1543" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1543" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Ranger Rick|HEALTH</v>
@@ -62756,7 +62739,7 @@
       </c>
       <c r="K1543" s="2"/>
     </row>
-    <row r="1544" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1544" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1544" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Ranger Rick|HOME</v>
@@ -62791,7 +62774,7 @@
       </c>
       <c r="K1544" s="2"/>
     </row>
-    <row r="1545" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1545" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1545" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Ranger Rick|JOB</v>
@@ -62826,7 +62809,7 @@
       </c>
       <c r="K1545" s="2"/>
     </row>
-    <row r="1546" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1546" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1546" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Ranger Rick|LOOK</v>
@@ -62861,7 +62844,7 @@
       </c>
       <c r="K1546" s="2"/>
     </row>
-    <row r="1547" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1547" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1547" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Ranger Rick|NAME</v>
@@ -62896,7 +62879,7 @@
       </c>
       <c r="K1547" s="2"/>
     </row>
-    <row r="1548" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1548" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1548" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Ranger Rick|RANG</v>
@@ -62931,7 +62914,7 @@
       </c>
       <c r="K1548" s="2"/>
     </row>
-    <row r="1549" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1549" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1549" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Short Round|HEALTH</v>
@@ -62966,7 +62949,7 @@
       </c>
       <c r="K1549" s="2"/>
     </row>
-    <row r="1550" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1550" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1550" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Short Round|JOB</v>
@@ -63001,7 +62984,7 @@
       </c>
       <c r="K1550" s="2"/>
     </row>
-    <row r="1551" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1551" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1551" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Short Round|JONE</v>
@@ -63036,7 +63019,7 @@
       </c>
       <c r="K1551" s="2"/>
     </row>
-    <row r="1552" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1552" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1552" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Short Round|LOOK</v>
@@ -63071,7 +63054,7 @@
       </c>
       <c r="K1552" s="2"/>
     </row>
-    <row r="1553" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1553" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1553" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Short Round|NAME</v>
@@ -63106,7 +63089,7 @@
       </c>
       <c r="K1553" s="2"/>
     </row>
-    <row r="1554" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1554" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1554" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Short Round|QUES</v>
@@ -63141,7 +63124,7 @@
       </c>
       <c r="K1554" s="2"/>
     </row>
-    <row r="1555" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1555" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1555" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Cy Lent|BEH</v>
@@ -63170,7 +63153,7 @@
       <c r="J1555" s="2"/>
       <c r="K1555" s="2"/>
     </row>
-    <row r="1556" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1556" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1556" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Cy Lent|HEALTH</v>
@@ -63199,7 +63182,7 @@
       <c r="J1556" s="2"/>
       <c r="K1556" s="2"/>
     </row>
-    <row r="1557" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1557" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1557" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Cy Lent|JOB</v>
@@ -63228,7 +63211,7 @@
       <c r="J1557" s="2"/>
       <c r="K1557" s="2"/>
     </row>
-    <row r="1558" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1558" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1558" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Cy Lent|LOOK</v>
@@ -63257,7 +63240,7 @@
       <c r="J1558" s="2"/>
       <c r="K1558" s="2"/>
     </row>
-    <row r="1559" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1559" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1559" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Cy Lent|NAME</v>
@@ -63286,7 +63269,7 @@
       <c r="J1559" s="2"/>
       <c r="K1559" s="2"/>
     </row>
-    <row r="1560" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1560" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1560" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Talfourd|HEALTH</v>
@@ -63323,7 +63306,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1561" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1561" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1561" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Talfourd|JOB</v>
@@ -63360,7 +63343,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1562" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1562" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1562" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Talfourd|JUST</v>
@@ -63397,7 +63380,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1563" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1563" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1563" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Talfourd|LOOK</v>
@@ -63434,7 +63417,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1564" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1564" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1564" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Talfourd|NAME</v>
@@ -63471,7 +63454,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1565" spans="1:11" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1565" spans="1:11" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A1565" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Talfourd|RUNE</v>
@@ -63508,7 +63491,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="1566" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1566" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1566" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Vorpal|HEALTH</v>
@@ -63543,7 +63526,7 @@
       </c>
       <c r="K1566" s="2"/>
     </row>
-    <row r="1567" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1567" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1567" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Vorpal|JOB</v>
@@ -63578,7 +63561,7 @@
       </c>
       <c r="K1567" s="2"/>
     </row>
-    <row r="1568" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1568" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1568" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Vorpal|LOOK</v>
@@ -63613,7 +63596,7 @@
       </c>
       <c r="K1568" s="2"/>
     </row>
-    <row r="1569" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1569" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1569" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Vorpal|NAME</v>
@@ -63648,7 +63631,7 @@
       </c>
       <c r="K1569" s="2"/>
     </row>
-    <row r="1570" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1570" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1570" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Vorpal|PEOP</v>
@@ -63683,7 +63666,7 @@
       </c>
       <c r="K1570" s="2"/>
     </row>
-    <row r="1571" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1571" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1571" t="str">
         <f t="shared" si="24"/>
         <v>Yew|Vorpal|VILL</v>
@@ -64065,13 +64048,13 @@
         <v>277</v>
       </c>
       <c r="D1610" s="2" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
       <c r="E1610" s="2" t="s">
         <v>16</v>
       </c>
       <c r="F1610" s="2" t="s">
-        <v>2632</v>
+        <v>2631</v>
       </c>
     </row>
   </sheetData>
@@ -64079,6 +64062,10 @@
     <filterColumn colId="2">
       <filters>
         <filter val="Lycaeum"/>
+        <filter val="Magincia"/>
+        <filter val="Minoc"/>
+        <filter val="Skara Brae"/>
+        <filter val="Yew"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3">
@@ -64130,7 +64117,7 @@
         <v>2444</v>
       </c>
       <c r="H1" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
@@ -65547,7 +65534,7 @@
         <v>A withering soul</v>
       </c>
       <c r="D54" s="50" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
       <c r="E54" s="19" t="str">
         <f t="shared" si="19"/>
@@ -65582,7 +65569,7 @@
         <v>A beautiful mage</v>
       </c>
       <c r="D55" s="50" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="E55" s="19" t="str">
         <f t="shared" si="19"/>
@@ -65617,7 +65604,7 @@
         <v>A noble fighter.</v>
       </c>
       <c r="D56" s="50" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="E56" s="19" t="str">
         <f t="shared" si="19"/>
@@ -65652,7 +65639,7 @@
         <v>A strange person</v>
       </c>
       <c r="D57" s="50" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="E57" s="19" t="str">
         <f t="shared" si="19"/>
@@ -65928,10 +65915,10 @@
         <v>1001</v>
       </c>
       <c r="B66" s="52" t="s">
-        <v>2573</v>
+        <v>2572</v>
       </c>
       <c r="C66" s="52" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="D66" s="50" t="s">
         <v>2514</v>
@@ -65969,7 +65956,7 @@
         <v>A valiant warrior.</v>
       </c>
       <c r="D67" s="50" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
       <c r="E67" s="19" t="str">
         <f t="shared" ref="E67:E68" si="23">"/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"""&amp;B67&amp;"""}"</f>
@@ -65997,10 +65984,10 @@
         <v>1514</v>
       </c>
       <c r="B68" s="22" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
       <c r="C68" s="61" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D68" s="50" t="s">
         <v>2507</v>
@@ -66031,13 +66018,13 @@
         <v>1514</v>
       </c>
       <c r="B69" s="52" t="s">
-        <v>2579</v>
+        <v>2578</v>
       </c>
       <c r="C69" s="58" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
       <c r="D69" s="50" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
       <c r="E69" s="19" t="str">
         <f t="shared" ref="E69:E73" si="25">"/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"""&amp;B69&amp;"""}"</f>
@@ -66065,13 +66052,13 @@
         <v>1514</v>
       </c>
       <c r="B70" s="52" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="C70" s="58" t="s">
-        <v>2583</v>
+        <v>2582</v>
       </c>
       <c r="D70" s="50" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
       <c r="E70" s="19" t="str">
         <f t="shared" si="25"/>
@@ -66102,7 +66089,7 @@
         <v>848</v>
       </c>
       <c r="C71" s="58" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
       <c r="E71" s="19" t="str">
         <f t="shared" si="25"/>
@@ -66130,13 +66117,13 @@
         <v>1514</v>
       </c>
       <c r="B72" s="65" t="s">
+        <v>2590</v>
+      </c>
+      <c r="C72" s="65" t="s">
         <v>2591</v>
       </c>
-      <c r="C72" s="65" t="s">
+      <c r="D72" s="67" t="s">
         <v>2592</v>
-      </c>
-      <c r="D72" s="67" t="s">
-        <v>2593</v>
       </c>
       <c r="E72" s="19" t="str">
         <f>"/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"""&amp;B72&amp;"""}"</f>
@@ -66171,7 +66158,7 @@
         <v>A grimy beggar.</v>
       </c>
       <c r="D73" s="50" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
       <c r="E73" s="19" t="str">
         <f t="shared" si="25"/>
@@ -66202,10 +66189,10 @@
         <v>1631</v>
       </c>
       <c r="C74" s="65" t="s">
+        <v>2594</v>
+      </c>
+      <c r="D74" s="66" t="s">
         <v>2595</v>
-      </c>
-      <c r="D74" s="66" t="s">
-        <v>2596</v>
       </c>
       <c r="E74" s="19" t="str">
         <f t="shared" ref="E74:E81" si="30">"/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"""&amp;B74&amp;"""}"</f>
@@ -66240,7 +66227,7 @@
         <v>An injured man.</v>
       </c>
       <c r="D75" s="50" t="s">
-        <v>2586</v>
+        <v>2585</v>
       </c>
       <c r="E75" s="19" t="str">
         <f t="shared" si="30"/>
@@ -66275,7 +66262,7 @@
         <v>A hungry beggar.</v>
       </c>
       <c r="D76" s="50" t="s">
-        <v>2594</v>
+        <v>2593</v>
       </c>
       <c r="E76" s="19" t="str">
         <f t="shared" si="30"/>
@@ -66310,7 +66297,7 @@
         <v>A ghostly figure</v>
       </c>
       <c r="D77" s="70" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="E77" s="19" t="str">
         <f t="shared" si="30"/>
@@ -66345,7 +66332,7 @@
         <v>A very small wizard.</v>
       </c>
       <c r="D78" s="50" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
       <c r="E78" s="19" t="str">
         <f t="shared" si="30"/>
@@ -66380,7 +66367,7 @@
         <v>A short dumpy man with a book.</v>
       </c>
       <c r="D79" s="50" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E79" s="19" t="str">
         <f t="shared" si="30"/>
@@ -66415,7 +66402,7 @@
         <v>A tall ranger.</v>
       </c>
       <c r="D80" s="50" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="E80" s="19" t="str">
         <f t="shared" si="30"/>
@@ -66450,7 +66437,7 @@
         <v>A solemn ranger.</v>
       </c>
       <c r="D81" s="50" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="E81" s="19" t="str">
         <f t="shared" si="30"/>
@@ -66520,7 +66507,7 @@
         <v>A tinker at the table.</v>
       </c>
       <c r="D83" s="50" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
       <c r="E83" s="19" t="str">
         <f t="shared" si="35"/>
@@ -66814,7 +66801,7 @@
         <v>A rotund tinker.</v>
       </c>
       <c r="D92" s="50" t="s">
-        <v>2611</v>
+        <v>2610</v>
       </c>
       <c r="E92" s="19" t="str">
         <f t="shared" si="35"/>
@@ -66849,7 +66836,7 @@
         <v>A cute bard.</v>
       </c>
       <c r="D93" s="50" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
       <c r="E93" s="19" t="str">
         <f t="shared" si="35"/>
@@ -66912,7 +66899,7 @@
         <v>316</v>
       </c>
       <c r="C95" s="52" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="E95" s="19" t="str">
         <f t="shared" si="35"/>
@@ -66940,13 +66927,13 @@
         <v>1130</v>
       </c>
       <c r="B96" s="52" t="s">
+        <v>2602</v>
+      </c>
+      <c r="C96" s="52" t="s">
         <v>2603</v>
       </c>
-      <c r="C96" s="52" t="s">
-        <v>2604</v>
-      </c>
       <c r="D96" s="50" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
       <c r="E96" s="19" t="str">
         <f t="shared" si="35"/>
@@ -66974,10 +66961,10 @@
         <v>1130</v>
       </c>
       <c r="B97" s="65" t="s">
+        <v>2606</v>
+      </c>
+      <c r="C97" s="65" t="s">
         <v>2607</v>
-      </c>
-      <c r="C97" s="65" t="s">
-        <v>2608</v>
       </c>
       <c r="D97" s="67" t="s">
         <v>2507</v>
@@ -67008,10 +66995,10 @@
         <v>1130</v>
       </c>
       <c r="B98" s="52" t="s">
-        <v>2613</v>
+        <v>2612</v>
       </c>
       <c r="C98" s="52" t="s">
-        <v>2615</v>
+        <v>2614</v>
       </c>
       <c r="D98" s="50" t="s">
         <v>2512</v>
@@ -67042,10 +67029,10 @@
         <v>1130</v>
       </c>
       <c r="B99" s="52" t="s">
-        <v>2614</v>
+        <v>2613</v>
       </c>
       <c r="C99" s="52" t="s">
-        <v>2617</v>
+        <v>2616</v>
       </c>
       <c r="D99" s="50" t="s">
         <v>2511</v>
@@ -67076,7 +67063,7 @@
         <v>858</v>
       </c>
       <c r="B100" s="22" t="s">
-        <v>2618</v>
+        <v>2617</v>
       </c>
       <c r="C100" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A100&amp;"|"&amp;B100&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A100&amp;"|"&amp;B100&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A100&amp;"|"&amp;B100&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67204,7 +67191,7 @@
         <v>858</v>
       </c>
       <c r="B104" s="22" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
       <c r="C104" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A104&amp;"|"&amp;B104&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A104&amp;"|"&amp;B104&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A104&amp;"|"&amp;B104&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67428,7 +67415,7 @@
         <v>858</v>
       </c>
       <c r="B111" s="22" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="C111" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A111&amp;"|"&amp;B111&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A111&amp;"|"&amp;B111&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A111&amp;"|"&amp;B111&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67460,7 +67447,7 @@
         <v>858</v>
       </c>
       <c r="B112" s="22" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="C112" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A112&amp;"|"&amp;B112&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A112&amp;"|"&amp;B112&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A112&amp;"|"&amp;B112&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67492,7 +67479,7 @@
         <v>858</v>
       </c>
       <c r="B113" s="22" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
       <c r="C113" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A113&amp;"|"&amp;B113&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A113&amp;"|"&amp;B113&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A113&amp;"|"&amp;B113&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67524,7 +67511,7 @@
         <v>858</v>
       </c>
       <c r="B114" s="22" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="C114" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A114&amp;"|"&amp;B114&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A114&amp;"|"&amp;B114&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A114&amp;"|"&amp;B114&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67556,7 +67543,7 @@
         <v>858</v>
       </c>
       <c r="B115" s="22" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
       <c r="C115" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A115&amp;"|"&amp;B115&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A115&amp;"|"&amp;B115&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A115&amp;"|"&amp;B115&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67588,7 +67575,7 @@
         <v>858</v>
       </c>
       <c r="B116" s="22" t="s">
-        <v>2624</v>
+        <v>2623</v>
       </c>
       <c r="C116" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A116&amp;"|"&amp;B116&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A116&amp;"|"&amp;B116&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A116&amp;"|"&amp;B116&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67620,7 +67607,7 @@
         <v>858</v>
       </c>
       <c r="B117" s="22" t="s">
-        <v>2625</v>
+        <v>2624</v>
       </c>
       <c r="C117" s="72" t="e">
         <f>IF(ISNA(VLOOKUP(A117&amp;"|"&amp;B117&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A117&amp;"|"&amp;B117&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A117&amp;"|"&amp;B117&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
@@ -67659,7 +67646,7 @@
         <v>A tall ghost.</v>
       </c>
       <c r="D118" s="50" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
       <c r="E118" s="19" t="str">
         <f t="shared" si="40"/>
@@ -67799,7 +67786,7 @@
         <v>A horrible ghastly devil!</v>
       </c>
       <c r="D122" s="50" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="E122" s="19" t="str">
         <f t="shared" si="40"/>
@@ -67823,7 +67810,7 @@
       </c>
     </row>
     <row r="123" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A123" s="77" t="s">
+      <c r="A123" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B123" s="52" t="s">
@@ -67833,30 +67820,29 @@
         <f>IF(ISNA(VLOOKUP(A123&amp;"|"&amp;B123&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A123&amp;"|"&amp;B123&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A123&amp;"|"&amp;B123&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A charming lady</v>
       </c>
-      <c r="D123" s="79"/>
-      <c r="E123" s="80" t="str">
+      <c r="E123" s="19" t="str">
         <f t="shared" si="40"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Beth Frasier"}</v>
       </c>
-      <c r="F123" s="78" t="str">
+      <c r="F123" s="22" t="str">
         <f t="shared" si="41"/>
         <v>/tag @e[type=minecraft:villager,name="Beth Frasier",limit=1] add npc_beth_frasier</v>
       </c>
-      <c r="G123" s="81" t="str">
+      <c r="G123" t="str">
         <f t="shared" si="42"/>
         <v>Beth Frasier</v>
       </c>
-      <c r="H123" s="81" t="str">
+      <c r="H123" t="str">
         <f t="shared" si="43"/>
         <v>npc_beth_frasier</v>
       </c>
-      <c r="I123" s="81">
+      <c r="I123">
         <f t="shared" si="44"/>
         <v>62</v>
       </c>
     </row>
     <row r="124" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A124" s="77" t="s">
+      <c r="A124" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B124" s="52" t="s">
@@ -67866,32 +67852,32 @@
         <f>IF(ISNA(VLOOKUP(A124&amp;"|"&amp;B124&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A124&amp;"|"&amp;B124&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A124&amp;"|"&amp;B124&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A short druid</v>
       </c>
-      <c r="D124" s="79" t="s">
-        <v>2638</v>
-      </c>
-      <c r="E124" s="80" t="str">
+      <c r="D124" s="50" t="s">
+        <v>2637</v>
+      </c>
+      <c r="E124" s="19" t="str">
         <f t="shared" ref="E124:E133" si="45">"/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"""&amp;B124&amp;"""}"</f>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Estro"}</v>
       </c>
-      <c r="F124" s="78" t="str">
+      <c r="F124" s="22" t="str">
         <f t="shared" ref="F124:F133" si="46">"/tag @e[type=minecraft:villager,name="""&amp;B124&amp;""",limit=1] add npc_"&amp;SUBSTITUTE(LOWER(B124)," ","_")</f>
         <v>/tag @e[type=minecraft:villager,name="Estro",limit=1] add npc_estro</v>
       </c>
-      <c r="G124" s="81" t="str">
+      <c r="G124" t="str">
         <f t="shared" ref="G124:G133" si="47">B124</f>
         <v>Estro</v>
       </c>
-      <c r="H124" s="81" t="str">
+      <c r="H124" t="str">
         <f t="shared" ref="H124:H133" si="48">MID(F124,I124+4,99)</f>
         <v>npc_estro</v>
       </c>
-      <c r="I124" s="81">
+      <c r="I124">
         <f t="shared" ref="I124:I133" si="49">FIND("add npc",F124)</f>
         <v>55</v>
       </c>
     </row>
     <row r="125" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A125" s="77" t="s">
+      <c r="A125" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B125" s="52" t="s">
@@ -67901,32 +67887,32 @@
         <f>IF(ISNA(VLOOKUP(A125&amp;"|"&amp;B125&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A125&amp;"|"&amp;B125&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A125&amp;"|"&amp;B125&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>An old druid, who looks strangely familiar.</v>
       </c>
-      <c r="D125" s="79" t="s">
-        <v>2633</v>
-      </c>
-      <c r="E125" s="80" t="str">
+      <c r="D125" s="50" t="s">
+        <v>2632</v>
+      </c>
+      <c r="E125" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Father Antos"}</v>
       </c>
-      <c r="F125" s="78" t="str">
+      <c r="F125" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Father Antos",limit=1] add npc_father_antos</v>
       </c>
-      <c r="G125" s="81" t="str">
+      <c r="G125" t="str">
         <f t="shared" si="47"/>
         <v>Father Antos</v>
       </c>
-      <c r="H125" s="81" t="str">
+      <c r="H125" t="str">
         <f t="shared" si="48"/>
         <v>npc_father_antos</v>
       </c>
-      <c r="I125" s="81">
+      <c r="I125">
         <f t="shared" si="49"/>
         <v>62</v>
       </c>
     </row>
     <row r="126" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A126" s="77" t="s">
+      <c r="A126" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B126" s="52" t="s">
@@ -67936,32 +67922,32 @@
         <f>IF(ISNA(VLOOKUP(A126&amp;"|"&amp;B126&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A126&amp;"|"&amp;B126&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A126&amp;"|"&amp;B126&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A tall agile man</v>
       </c>
-      <c r="D126" s="79" t="s">
-        <v>2637</v>
-      </c>
-      <c r="E126" s="80" t="str">
+      <c r="D126" s="50" t="s">
+        <v>2636</v>
+      </c>
+      <c r="E126" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Lord Terence"}</v>
       </c>
-      <c r="F126" s="78" t="str">
+      <c r="F126" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Lord Terence",limit=1] add npc_lord_terence</v>
       </c>
-      <c r="G126" s="81" t="str">
+      <c r="G126" t="str">
         <f t="shared" si="47"/>
         <v>Lord Terence</v>
       </c>
-      <c r="H126" s="81" t="str">
+      <c r="H126" t="str">
         <f t="shared" si="48"/>
         <v>npc_lord_terence</v>
       </c>
-      <c r="I126" s="81">
+      <c r="I126">
         <f t="shared" si="49"/>
         <v>62</v>
       </c>
     </row>
     <row r="127" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A127" s="77" t="s">
+      <c r="A127" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B127" s="52" t="s">
@@ -67971,30 +67957,29 @@
         <f>IF(ISNA(VLOOKUP(A127&amp;"|"&amp;B127&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A127&amp;"|"&amp;B127&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A127&amp;"|"&amp;B127&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A noble wizard</v>
       </c>
-      <c r="D127" s="79"/>
-      <c r="E127" s="80" t="str">
+      <c r="E127" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Nigel"}</v>
       </c>
-      <c r="F127" s="78" t="str">
+      <c r="F127" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Nigel",limit=1] add npc_nigel</v>
       </c>
-      <c r="G127" s="81" t="str">
+      <c r="G127" t="str">
         <f t="shared" si="47"/>
         <v>Nigel</v>
       </c>
-      <c r="H127" s="81" t="str">
+      <c r="H127" t="str">
         <f t="shared" si="48"/>
         <v>npc_nigel</v>
       </c>
-      <c r="I127" s="81">
+      <c r="I127">
         <f t="shared" si="49"/>
         <v>55</v>
       </c>
     </row>
     <row r="128" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A128" s="77" t="s">
+      <c r="A128" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B128" s="52" t="s">
@@ -68004,65 +67989,64 @@
         <f>IF(ISNA(VLOOKUP(A128&amp;"|"&amp;B128&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A128&amp;"|"&amp;B128&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A128&amp;"|"&amp;B128&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A stately baron</v>
       </c>
-      <c r="D128" s="79"/>
-      <c r="E128" s="80" t="str">
+      <c r="E128" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Robert Frasier"}</v>
       </c>
-      <c r="F128" s="78" t="str">
+      <c r="F128" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Robert Frasier",limit=1] add npc_robert_frasier</v>
       </c>
-      <c r="G128" s="81" t="str">
+      <c r="G128" t="str">
         <f t="shared" si="47"/>
         <v>Robert Frasier</v>
       </c>
-      <c r="H128" s="81" t="str">
+      <c r="H128" t="str">
         <f t="shared" si="48"/>
         <v>npc_robert_frasier</v>
       </c>
-      <c r="I128" s="81">
+      <c r="I128">
         <f t="shared" si="49"/>
         <v>64</v>
       </c>
     </row>
     <row r="129" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A129" s="77" t="s">
+      <c r="A129" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B129" s="52" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
       <c r="C129" s="53" t="str">
         <f>IF(ISNA(VLOOKUP(A129&amp;"|"&amp;B129&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A129&amp;"|"&amp;B129&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A129&amp;"|"&amp;B129&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A tall mage wearing strange armour.</v>
       </c>
       <c r="D129" s="50" t="s">
-        <v>2634</v>
-      </c>
-      <c r="E129" s="80" t="str">
+        <v>2633</v>
+      </c>
+      <c r="E129" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Scatuu"}</v>
       </c>
-      <c r="F129" s="78" t="str">
+      <c r="F129" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Scatuu",limit=1] add npc_scatuu</v>
       </c>
-      <c r="G129" s="81" t="str">
+      <c r="G129" t="str">
         <f t="shared" si="47"/>
         <v>Scatuu</v>
       </c>
-      <c r="H129" s="81" t="str">
+      <c r="H129" t="str">
         <f t="shared" si="48"/>
         <v>npc_scatuu</v>
       </c>
-      <c r="I129" s="81">
+      <c r="I129">
         <f t="shared" si="49"/>
         <v>56</v>
       </c>
     </row>
     <row r="130" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A130" s="77" t="s">
+      <c r="A130" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B130" s="52" t="s">
@@ -68072,62 +68056,61 @@
         <f>IF(ISNA(VLOOKUP(A130&amp;"|"&amp;B130&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A130&amp;"|"&amp;B130&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A130&amp;"|"&amp;B130&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A pitiful beggar</v>
       </c>
-      <c r="E130" s="80" t="str">
+      <c r="E130" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Shylock the Meek"}</v>
       </c>
-      <c r="F130" s="78" t="str">
+      <c r="F130" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Shylock the Meek",limit=1] add npc_shylock_the_meek</v>
       </c>
-      <c r="G130" s="81" t="str">
+      <c r="G130" t="str">
         <f t="shared" si="47"/>
         <v>Shylock the Meek</v>
       </c>
-      <c r="H130" s="81" t="str">
+      <c r="H130" t="str">
         <f t="shared" si="48"/>
         <v>npc_shylock_the_meek</v>
       </c>
-      <c r="I130" s="81">
+      <c r="I130">
         <f t="shared" si="49"/>
         <v>66</v>
       </c>
     </row>
     <row r="131" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A131" s="77" t="s">
+      <c r="A131" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B131" s="52" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
       <c r="C131" s="53" t="str">
         <f>IF(ISNA(VLOOKUP(A131&amp;"|"&amp;B131&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A131&amp;"|"&amp;B131&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A131&amp;"|"&amp;B131&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>Proprietor of The Truth Healer</v>
       </c>
-      <c r="D131" s="79"/>
-      <c r="E131" s="80" t="str">
+      <c r="E131" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Starfire"}</v>
       </c>
-      <c r="F131" s="78" t="str">
+      <c r="F131" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Starfire",limit=1] add npc_starfire</v>
       </c>
-      <c r="G131" s="81" t="str">
+      <c r="G131" t="str">
         <f t="shared" si="47"/>
         <v>Starfire</v>
       </c>
-      <c r="H131" s="81" t="str">
+      <c r="H131" t="str">
         <f t="shared" si="48"/>
         <v>npc_starfire</v>
       </c>
-      <c r="I131" s="81">
+      <c r="I131">
         <f t="shared" si="49"/>
         <v>58</v>
       </c>
     </row>
     <row r="132" spans="1:9" ht="21.6" x14ac:dyDescent="0.3">
-      <c r="A132" s="77" t="s">
+      <c r="A132" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B132" s="52" t="s">
@@ -68137,42 +68120,42 @@
         <f>IF(ISNA(VLOOKUP(A132&amp;"|"&amp;B132&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE)),VLOOKUP(A132&amp;"|"&amp;B132&amp;"|"&amp;"You see..",'NPC Dialogue'!$A:$F,6,FALSE),VLOOKUP(A132&amp;"|"&amp;B132&amp;"|"&amp;"LOOK",'NPC Dialogue'!$A:$F,6,FALSE))</f>
         <v>A stately wizard</v>
       </c>
-      <c r="D132" s="79" t="s">
-        <v>2572</v>
-      </c>
-      <c r="E132" s="80" t="str">
+      <c r="D132" s="50" t="s">
+        <v>2571</v>
+      </c>
+      <c r="E132" s="19" t="str">
         <f t="shared" si="45"/>
         <v>/data merge entity @e[type=minecraft:villager,limit=1,sort=nearest] {CustomName:"Tymus"}</v>
       </c>
-      <c r="F132" s="78" t="str">
+      <c r="F132" s="22" t="str">
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Tymus",limit=1] add npc_tymus</v>
       </c>
-      <c r="G132" s="81" t="str">
+      <c r="G132" t="str">
         <f t="shared" si="47"/>
         <v>Tymus</v>
       </c>
-      <c r="H132" s="81" t="str">
+      <c r="H132" t="str">
         <f t="shared" si="48"/>
         <v>npc_tymus</v>
       </c>
-      <c r="I132" s="81">
+      <c r="I132">
         <f t="shared" si="49"/>
         <v>55</v>
       </c>
     </row>
     <row r="133" spans="1:9" ht="42" x14ac:dyDescent="0.3">
-      <c r="A133" s="77" t="s">
+      <c r="A133" s="20" t="s">
         <v>277</v>
       </c>
       <c r="B133" s="52" t="s">
+        <v>2638</v>
+      </c>
+      <c r="C133" s="52" t="s">
         <v>2639</v>
       </c>
-      <c r="C133" s="52" t="s">
+      <c r="D133" s="50" t="s">
         <v>2640</v>
-      </c>
-      <c r="D133" s="50" t="s">
-        <v>2641</v>
       </c>
       <c r="E133" s="19" t="str">
         <f t="shared" si="45"/>
@@ -68182,15 +68165,15 @@
         <f t="shared" si="46"/>
         <v>/tag @e[type=minecraft:villager,name="Nearly A Corpse",limit=1] add npc_nearly_a_corpse</v>
       </c>
-      <c r="G133" s="81" t="str">
+      <c r="G133" t="str">
         <f t="shared" si="47"/>
         <v>Nearly A Corpse</v>
       </c>
-      <c r="H133" s="81" t="str">
+      <c r="H133" t="str">
         <f t="shared" si="48"/>
         <v>npc_nearly_a_corpse</v>
       </c>
-      <c r="I133" s="81">
+      <c r="I133">
         <f t="shared" si="49"/>
         <v>65</v>
       </c>
@@ -68270,7 +68253,7 @@
         <v>1001</v>
       </c>
       <c r="G8" s="47" t="s">
-        <v>2568</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -68278,7 +68261,7 @@
         <v>277</v>
       </c>
       <c r="G10" s="47" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
@@ -68287,12 +68270,12 @@
       </c>
       <c r="D11" s="74"/>
       <c r="F11" s="74" t="s">
-        <v>2629</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B13" s="73" t="s">
-        <v>2627</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="26.4" x14ac:dyDescent="0.3">
@@ -70327,7 +70310,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="str">
         <f t="shared" si="1"/>
         <v>Towns|Moonglow|Patric the Humble Shepherd|HUMI</v>
@@ -72637,7 +72620,7 @@
         <v>1719</v>
       </c>
     </row>
-    <row r="181" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" t="str">
         <f t="shared" si="2"/>
         <v>Towns|Magincia|Bulbous|SPOI</v>

</xml_diff>

<commit_message>
Minoc trades and conversations - most of them. Need to do innkeeper, room rental, and forge iron door mechanic.
</commit_message>
<xml_diff>
--- a/spoilers/Ultima_IV_NPC_Dialogue_COMPLETE-with-MC.xlsx
+++ b/spoilers/Ultima_IV_NPC_Dialogue_COMPLETE-with-MC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A09859-48BF-46DA-A13D-9371047369AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA9A2E3-3CB2-42B2-BC59-2FD32ED59E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" tabRatio="728" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,13 @@
     <sheet name="NPC Dialogue" sheetId="1" r:id="rId1"/>
     <sheet name="MC-NPC_TAGS" sheetId="8" r:id="rId2"/>
     <sheet name="gameDesignMisc" sheetId="10" r:id="rId3"/>
-    <sheet name="UsefulTagCmds" sheetId="9" r:id="rId4"/>
-    <sheet name="Runes_Stones_Mantras" sheetId="5" r:id="rId5"/>
-    <sheet name="QuestionTriggers" sheetId="4" r:id="rId6"/>
-    <sheet name="MC-InterTownDependencies" sheetId="7" r:id="rId7"/>
-    <sheet name="TheGypsy" sheetId="3" r:id="rId8"/>
-    <sheet name="Barkeeps" sheetId="2" r:id="rId9"/>
+    <sheet name="game_findingOtherTowns" sheetId="11" r:id="rId4"/>
+    <sheet name="UsefulTagCmds" sheetId="9" r:id="rId5"/>
+    <sheet name="Runes_Stones_Mantras" sheetId="5" r:id="rId6"/>
+    <sheet name="QuestionTriggers" sheetId="4" r:id="rId7"/>
+    <sheet name="MC-InterTownDependencies" sheetId="7" r:id="rId8"/>
+    <sheet name="TheGypsy" sheetId="3" r:id="rId9"/>
+    <sheet name="Barkeeps" sheetId="2" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MC-NPC_TAGS'!$A$1:$F$123</definedName>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14365" uniqueCount="2644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14408" uniqueCount="2666">
   <si>
     <t>town_type</t>
   </si>
@@ -8248,6 +8249,72 @@
   </si>
   <si>
     <t>Has 1-2 of the three metallurgists</t>
+  </si>
+  <si>
+    <t>one is near a woodland's monument (possibly jhelom)</t>
+  </si>
+  <si>
+    <t>3 towns are lined up North-South with stone circle  (Lycaeum, Skara Brae, Britain)</t>
+  </si>
+  <si>
+    <t>2 towns are lined up East-West (Jhelom …and stone circle ...and …. _&lt;moongate to end_game&gt;…?)</t>
+  </si>
+  <si>
+    <t>some towns are in biomes (eg savannah, desert)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">savannah: </t>
+  </si>
+  <si>
+    <t>magincia</t>
+  </si>
+  <si>
+    <t>moonglow</t>
+  </si>
+  <si>
+    <t>desert:</t>
+  </si>
+  <si>
+    <t>trinsic</t>
+  </si>
+  <si>
+    <t>minoc</t>
+  </si>
+  <si>
+    <t>dark oak:</t>
+  </si>
+  <si>
+    <t>yew</t>
+  </si>
+  <si>
+    <t>spruce forest:</t>
+  </si>
+  <si>
+    <t>mycelium, mushrooms</t>
+  </si>
+  <si>
+    <t>Perhaps as mechanic to see forge, armor stand needs to be decked out with all-copper or all-iron or all-gold armor.  (expensive to purchase around the land, but basically tests METALLURGY granted)</t>
+  </si>
+  <si>
+    <t>Zircon in Minoc has all 3 books on METALLURGY (but you must already have 1 to get to see him)</t>
+  </si>
+  <si>
+    <t>Zircon has fire protection potion as a trade but you need to give him ____ for it (something that would be a SACRIFICE to give away).</t>
+  </si>
+  <si>
+    <t>After zircon says "ask at counter" (for weapons) then the counter offers MYSTIC (Magic) Armor</t>
+  </si>
+  <si>
+    <t>Zircon should say something about the VIRTUE of SACRIFICE.</t>
+  </si>
+  <si>
+    <t>REMOVE button to open iron door to get into forge</t>
+  </si>
+  <si>
+    <t>_Mechanics_</t>
+  </si>
+  <si>
+    <t>Forge</t>
   </si>
 </sst>
 </file>
@@ -64081,6 +64148,190 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CE45335-4D2B-4772-B0DD-9F9A6B658097}">
+  <sheetPr>
+    <tabColor theme="1"/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5546875" customWidth="1"/>
+    <col min="5" max="5" width="44.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2351</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2277</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2278</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2279</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>858</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2277</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2280</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2281</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2277</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>2282</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>2283</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>2277</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>2284</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>2285</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>1768</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>1769</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2277</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>2286</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>2287</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>1768</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>2352</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>2277</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>2288</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>2289</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>1768</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>1890</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>2277</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>2290</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>2291</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{562612D2-39F9-45A4-AB64-E3ADF2A9E487}">
   <sheetPr>
@@ -68189,7 +68440,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="B3:G15"/>
+  <dimension ref="B3:G26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="41" customWidth="1"/>
@@ -68312,12 +68563,190 @@
         <v>1936</v>
       </c>
     </row>
+    <row r="18" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C18" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D18" t="s">
+        <v>2664</v>
+      </c>
+      <c r="F18" t="s">
+        <v>2658</v>
+      </c>
+    </row>
+    <row r="19" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E19" t="s">
+        <v>2665</v>
+      </c>
+      <c r="F19" t="s">
+        <v>2659</v>
+      </c>
+    </row>
+    <row r="20" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D20" t="s">
+        <v>1228</v>
+      </c>
+      <c r="F20" t="s">
+        <v>2660</v>
+      </c>
+    </row>
+    <row r="21" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C21" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1228</v>
+      </c>
+      <c r="F21" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="22" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1228</v>
+      </c>
+      <c r="F22" t="s">
+        <v>2662</v>
+      </c>
+    </row>
+    <row r="23" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D23" t="s">
+        <v>2664</v>
+      </c>
+      <c r="F23" t="s">
+        <v>2663</v>
+      </c>
+    </row>
+    <row r="24" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C24" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D24" t="s">
+        <v>2613</v>
+      </c>
+      <c r="E24" t="s">
+        <v>2511</v>
+      </c>
+    </row>
+    <row r="25" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D25" t="s">
+        <v>2613</v>
+      </c>
+      <c r="E25" t="s">
+        <v>2511</v>
+      </c>
+    </row>
+    <row r="26" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D26" t="s">
+        <v>2613</v>
+      </c>
+      <c r="E26" t="s">
+        <v>2511</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5114F14F-4C96-4F70-B8E1-5E940CA1DC1C}">
+  <dimension ref="B3:F14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>2646</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>2647</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>2648</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2649</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>2648</v>
+      </c>
+      <c r="D11" t="s">
+        <v>2650</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>2651</v>
+      </c>
+      <c r="D12" t="s">
+        <v>2652</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>2654</v>
+      </c>
+      <c r="D13" t="s">
+        <v>2655</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>2656</v>
+      </c>
+      <c r="D14" t="s">
+        <v>2653</v>
+      </c>
+      <c r="F14" t="s">
+        <v>2657</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53D045C2-8C8D-4A38-9694-9AED0BC2C885}">
   <sheetPr>
     <tabColor theme="1"/>
@@ -68375,7 +68804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{088C5635-A5EC-4122-84D7-6A89EEE95F11}">
   <sheetPr>
     <tabColor theme="2" tint="-0.499984740745262"/>
@@ -68825,7 +69254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{400D3863-610B-4E2B-A552-15E2A555CC9E}">
   <sheetPr>
     <tabColor theme="3" tint="0.39997558519241921"/>
@@ -73927,7 +74356,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E06EE1F-1C82-4E27-8E4C-F37AA3691D63}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -73977,7 +74406,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25C08808-B224-4412-8ADD-D4E58CA88804}">
   <sheetPr>
     <tabColor theme="1"/>
@@ -74621,188 +75050,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CE45335-4D2B-4772-B0DD-9F9A6B658097}">
-  <sheetPr>
-    <tabColor theme="1"/>
-  </sheetPr>
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5546875" customWidth="1"/>
-    <col min="5" max="5" width="44.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>2351</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>2278</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>2279</v>
-      </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>858</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2280</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2281</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>1001</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>2282</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>2283</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>1397</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>2284</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>2285</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>1768</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>1769</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>2286</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>2287</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>1768</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>2352</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>2288</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>2289</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>1768</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>1890</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>2277</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>2290</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>2291</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>